<commit_message>
Fix PDF extraction for Enrico analyzer
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Enrico_Deductions/enrico_deductions_monthly.xlsx
+++ b/08_Reports - Доклади - Berichte/Enrico_Deductions/enrico_deductions_monthly.xlsx
@@ -130,7 +130,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -420,12 +420,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t/>
+          <t>2.40</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t/>
+          <t>2.40</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -455,7 +455,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t/>
+          <t>2.40</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -465,17 +465,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t/>
+          <t>916.00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -532,17 +532,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -599,17 +599,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -621,12 +621,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -666,17 +666,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -688,12 +688,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t/>
+          <t>101.67</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -703,17 +703,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t/>
+          <t>1325.55</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t/>
+          <t>16.00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t/>
+          <t>1650.12</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -733,17 +733,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -755,12 +755,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t/>
+          <t>94.26</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t/>
+          <t>851.38</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t/>
+          <t>892.48</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -800,17 +800,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -822,12 +822,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -837,17 +837,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t/>
+          <t>532.49</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t/>
+          <t>16.00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t/>
+          <t>579.09</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -867,17 +867,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -889,12 +889,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t/>
+          <t>74.58</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -904,17 +904,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t/>
+          <t>1502.56</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t/>
+          <t>16.00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t/>
+          <t>1596.66</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -956,12 +956,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t/>
+          <t>32.44</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -971,17 +971,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t/>
+          <t>1060.60</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t/>
+          <t>16.00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t/>
+          <t>1075.27</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1001,17 +1001,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t/>
+          <t>2.50</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t/>
+          <t>16.00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t/>
+          <t>18.50</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.03</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.33</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1135,17 +1135,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve Enrico analyzer financial parsing
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Enrico_Deductions/enrico_deductions_monthly.xlsx
+++ b/08_Reports - Доклади - Berichte/Enrico_Deductions/enrico_deductions_monthly.xlsx
@@ -18,60 +18,85 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>gross_credit_total</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>gross_credit_gutschrift_total</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>abschlag_coincident_total</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>abschlag_mitnahme_total</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>abschlag_quittungslose_sendung_total</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>sendungsverlust_total</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>scannermiete_total</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>other_deductions_total</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>total_deductions</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>total_deductions_negative</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>refunds_total_positive</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>net_effect</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>net_amount_if_available</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>number_of_source_documents</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>missing_source_documents</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>source_document_numbers</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -130,15 +155,40 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
@@ -152,27 +202,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t/>
+          <t>186243.20</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t/>
+          <t>186243.20</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t/>
+          <t>-6245.92</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>-180.25</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t/>
+          <t>-123.00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -192,22 +242,47 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t/>
+          <t>-6549.17</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-6549.17</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t/>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>179694.03</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>7-2024</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -264,15 +339,40 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
@@ -331,15 +431,40 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
@@ -398,15 +523,40 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
@@ -420,12 +570,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t/>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t/>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -455,7 +605,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t/>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -465,17 +615,42 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t/>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
           <t/>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
       </c>
     </row>
@@ -487,62 +662,87 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>916.00</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>916.00</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>34-2024</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
       </c>
     </row>
@@ -554,12 +754,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t>176234.29</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>176234.29</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -569,7 +769,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -589,7 +789,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t/>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -599,15 +799,40 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>176234.29</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>31-2024</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -621,12 +846,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t>197442.02</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>197442.02</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -636,7 +861,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -656,7 +881,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t/>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -666,15 +891,40 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>197442.02</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>38-2024</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -688,12 +938,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>101.67</t>
+          <t>232318.76</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>232318.76</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -703,45 +953,70 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1325.55</t>
+          <t/>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>147.65</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>16.00</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1650.12</t>
+          <t/>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t/>
+          <t>163.65</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>232582.41</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>01999; 02000; 02001; 02002; 42-2024; 51-2025</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -755,12 +1030,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>94.26</t>
+          <t>188941.38</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>188941.38</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -770,17 +1045,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>851.38</t>
+          <t/>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t/>
+          <t>12.50</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -790,25 +1065,50 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>892.48</t>
+          <t/>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t/>
+          <t>12.50</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>95.95</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>189049.83</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>02014; 02015; 02023; 44-2024; 55-2025</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -822,12 +1122,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t>189578.90</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>189578.90</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -837,45 +1137,70 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>532.49</t>
+          <t/>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>51.89</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>16.00</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>579.09</t>
+          <t/>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t/>
+          <t>67.89</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>189646.79</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>02035; 02036; 02037; 02038; 48-2025</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -889,12 +1214,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>74.58</t>
+          <t>170271.25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>170271.25</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -904,45 +1229,70 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1502.56</t>
+          <t/>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>73.29</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>16.00</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1596.66</t>
+          <t/>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t/>
+          <t>89.29</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>75.91</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>170436.45</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>02054; 02055; 02056; 02057; 52-2025; 60-2025</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -956,12 +1306,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>32.44</t>
+          <t>202395.66</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>202395.66</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -971,45 +1321,70 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1060.60</t>
+          <t/>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>223.05</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>16.00</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1075.27</t>
+          <t/>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t/>
+          <t>239.05</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>202684.71</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>02068; 02069; 02070; 02766; 57-2025; 71-2025</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1043,40 +1418,65 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>2.50</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>16.00</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>18.50</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>18.50</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>02764; 02765; 02767</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>
@@ -1090,12 +1490,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t>120491.84</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>120491.84</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1105,7 +1505,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t/>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1125,7 +1525,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>-1.33</t>
+          <t/>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1135,15 +1535,40 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>120491.84</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>66-2025</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1202,15 +1627,40 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
         <is>
           <t>No Gutschrift/Abrechnung source document detected for this month.</t>
         </is>

</xml_diff>

<commit_message>
Refine Enrico missing month logic
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Enrico_Deductions/enrico_deductions_monthly.xlsx
+++ b/08_Reports - Доклади - Berichte/Enrico_Deductions/enrico_deductions_monthly.xlsx
@@ -88,15 +88,55 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>main_gutschrift_found</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>refunds_found</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>sendungsverlust_found</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>scanner_invoice_found</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>any_document_found</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>missing_main_monthly_gutschrift</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>has_only_refunds_or_corrections</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>has_any_enrico_document</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>missing_source_documents</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>source_document_numbers</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -180,17 +220,57 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t/>
+          <t>NO</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Enrico documents found, but no main monthly Gutschrift/Abrechnung detected.</t>
         </is>
       </c>
     </row>
@@ -272,17 +352,57 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
           <t>7-2024</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -364,17 +484,57 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t/>
+          <t>NO</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>No Enrico source document detected for this month.</t>
         </is>
       </c>
     </row>
@@ -456,17 +616,57 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t/>
+          <t>NO</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>No Enrico source document detected for this month.</t>
         </is>
       </c>
     </row>
@@ -548,17 +748,57 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t/>
+          <t>NO</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>No Enrico source document detected for this month.</t>
         </is>
       </c>
     </row>
@@ -640,17 +880,57 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t/>
+          <t>NO</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>No Enrico source document detected for this month.</t>
         </is>
       </c>
     </row>
@@ -732,17 +1012,57 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
           <t>34-2024</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Only refund/correction documents found; main monthly Gutschrift/Abrechnung is missing.</t>
         </is>
       </c>
     </row>
@@ -824,17 +1144,57 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
           <t>31-2024</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -916,17 +1276,57 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
           <t>38-2024</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1008,17 +1408,57 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
           <t>01999; 02000; 02001; 02002; 42-2024; 51-2025</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1100,17 +1540,57 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
           <t>02014; 02015; 02023; 44-2024; 55-2025</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1192,17 +1672,57 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
           <t>02035; 02036; 02037; 02038; 48-2025</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1284,17 +1804,57 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
           <t>02054; 02055; 02056; 02057; 52-2025; 60-2025</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1936,57 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
           <t>02068; 02069; 02070; 02766; 57-2025; 71-2025</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1468,17 +2068,57 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
           <t>02764; 02765; 02767</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Enrico documents found, but no main monthly Gutschrift/Abrechnung detected.</t>
         </is>
       </c>
     </row>
@@ -1560,17 +2200,57 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
           <t>66-2025</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t/>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Main monthly Gutschrift/Abrechnung found.</t>
         </is>
       </c>
     </row>
@@ -1652,17 +2332,57 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t/>
+          <t>NO</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>No Gutschrift/Abrechnung source document detected for this month.</t>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>No Enrico source document detected for this month.</t>
         </is>
       </c>
     </row>

</xml_diff>